<commit_message>
Simplifica los libros: una sola hoja y la tasa de mora publicada, sin IBC
Se elimina la columna del interes bancario corriente y las hojas Tasas y
Metodologia. Cada libro queda en una hoja: tramos por mes, dias, tasa de mora
publicada para ese mes, intereses y totales. La tasa de cada mes pasa a ser
celda editable dentro de la misma tabla.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017gU1GCSPt2rGeFm95WKPy5
</commit_message>
<xml_diff>
--- a/liquidaciones/Liquidacion_152646000_30abr2026_a_28may2026.xlsx
+++ b/liquidaciones/Liquidacion_152646000_30abr2026_a_28may2026.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Liquidacion" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tasas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Metodologia" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,15 +16,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="167" formatCode="0.000000%"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00;($#,##0.00);-"/>
-    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,24 +62,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00008000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
-      <color rgb="000000FF"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -135,25 +121,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,14 +148,7 @@
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,18 +514,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,7 +544,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Tasa de mora maxima legal (1,5 x IBC certificado por la Superfinanciera), mes a mes</t>
+          <t>Tasa de mora maxima legal publicada para cada mes de vigencia (art. 884 C.Co.)</t>
         </is>
       </c>
     </row>
@@ -587,11 +564,6 @@
       <c r="B6" s="5" t="n">
         <v>152646000</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Capital y fechas suministrados por el usuario.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -599,7 +571,7 @@
           <t>Fecha inicial de mora</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="6" t="n">
         <v>46142</v>
       </c>
     </row>
@@ -609,7 +581,7 @@
           <t>Fecha final de liquidacion</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="6" t="n">
         <v>46170</v>
       </c>
     </row>
@@ -619,152 +591,138 @@
           <t>Total dias de mora</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <f>B8-B7</f>
         <v/>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Mes de vigencia</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Desde</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Hasta</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Dias</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>IBC E.A.</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Tasa mora E.A.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Tasa diaria equiv.</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Intereses del periodo</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>Acto administrativo / observacion</t>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Fuente / observacion</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Abril 2026</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <v>46142</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="10" t="n">
         <v>46143</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <f>C12-B12</f>
         <v/>
       </c>
-      <c r="E12" s="12">
-        <f>Tasas!B5</f>
-        <v/>
+      <c r="E12" s="11" t="n">
+        <v>0.2676</v>
       </c>
       <c r="F12" s="12">
-        <f>Tasas!C5</f>
+        <f>(1+E12)^(1/365)-1</f>
         <v/>
       </c>
       <c r="G12" s="13">
-        <f>(1+F12)^(1/365)-1</f>
-        <v/>
-      </c>
-      <c r="H12" s="14">
-        <f>$B$6*((1+F12)^(D12/365)-1)</f>
-        <v/>
-      </c>
-      <c r="I12" s="15">
-        <f>Tasas!D5</f>
-        <v/>
+        <f>$B$6*((1+E12)^(D12/365)-1)</f>
+        <v/>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>Res. 0517 de 2026</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Mayo 2026</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="10" t="n">
         <v>46143</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="10" t="n">
         <v>46170</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="7">
         <f>C13-B13</f>
         <v/>
       </c>
-      <c r="E13" s="12">
-        <f>Tasas!B6</f>
-        <v/>
+      <c r="E13" s="11" t="n">
+        <v>0.2817</v>
       </c>
       <c r="F13" s="12">
-        <f>Tasas!C6</f>
+        <f>(1+E13)^(1/365)-1</f>
         <v/>
       </c>
       <c r="G13" s="13">
-        <f>(1+F13)^(1/365)-1</f>
-        <v/>
-      </c>
-      <c r="H13" s="14">
-        <f>$B$6*((1+F13)^(D13/365)-1)</f>
-        <v/>
-      </c>
-      <c r="I13" s="15">
-        <f>Tasas!D6</f>
-        <v/>
+        <f>$B$6*((1+E13)^(D13/365)-1)</f>
+        <v/>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Res. 0662 de 2026</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>TOTAL INTERESES DE MORA</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="18">
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="17">
         <f>SUM(D12:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="19">
-        <f>SUM(H12:H13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="17" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="18">
+        <f>SUM(G12:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -772,415 +730,53 @@
           <t>Capital</t>
         </is>
       </c>
-      <c r="H15" s="20">
+      <c r="G15" s="19">
         <f>$B$6</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>TOTAL A PAGAR (capital + intereses)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="22">
-        <f>H14+H15</f>
-        <v/>
-      </c>
-      <c r="I16" s="17" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="21">
+        <f>G14+G15</f>
+        <v/>
+      </c>
+      <c r="H16" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>- Formula de cada tramo: Capital x [ (1 + tasa mora E.A.) ^ (dias / 365) - 1 ].</t>
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>- Intereses de cada tramo = Capital x [ (1 + tasa mora E.A.) ^ (dias / 365) - 1 ].</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>- Los dias se cuentan como diferencia de fechas: se cuenta el dia inicial y no el final, de modo que el cambio de mes no duplica ningun dia.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>- Los intereses se calculan sobre el capital insoluto; no se capitalizan (no hay anatocismo).</t>
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>- Los intereses se liquidan sobre el capital insoluto; no se capitalizan (no hay anatocismo).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>- Celdas azules o amarillas: datos editables. Celdas verdes: traidas de la hoja Tasas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>- Detalle de tasas y fuentes en la hoja Tasas; supuestos y conteo en la hoja Metodologia.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1000"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tasas certificadas - Superintendencia Financiera de Colombia</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Credito de consumo y ordinario. Tasa de mora maxima legal = 1,5 x IBC (art. 884 C.Co.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Mes de vigencia</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>IBC E.A.</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Tasa mora E.A.</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Acto administrativo / observacion</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Abril 2026</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="n">
-        <v>0.1784</v>
-      </c>
-      <c r="C5" s="24">
-        <f>B5*$B$1000</f>
-        <v/>
-      </c>
-      <c r="D5" s="25" t="inlineStr">
-        <is>
-          <t>Resolucion 0517 de 2026 (27-mar-2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Mayo 2026</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="n">
-        <v>0.1878</v>
-      </c>
-      <c r="C6" s="24">
-        <f>B6*$B$1000</f>
-        <v/>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>Resolucion 0662 de 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: unicas editables.</t>
-        </is>
-      </c>
-    </row>
-    <row r="1000">
-      <c r="A1000" s="4" t="inlineStr">
-        <is>
-          <t>Factor legal de mora (1,5 veces el IBC)</t>
-        </is>
-      </c>
-      <c r="B1000" s="27" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C1000" s="3" t="inlineStr">
-        <is>
-          <t>Art. 884 Codigo de Comercio / art. 305 Codigo Penal (usura).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metodologia de la liquidacion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="28" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>1. Obligacion liquidada</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Capital: 152.646.000 pesos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Periodo de mora: 30/04/2026 a 28/05/2026 (28 dias).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Capital y fechas suministrados por el usuario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="28" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2. Tasa aplicada</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Se aplica, mes a mes, la tasa de mora maxima legal: 1,5 veces el Interes Bancario</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Corriente para credito de consumo y ordinario certificado por la Superintendencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Financiera de Colombia para cada mes de vigencia (art. 884 del Codigo de Comercio).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Esa tasa coincide con la tasa de usura certificada para la misma modalidad, de modo</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   que la liquidacion no excede el limite del art. 305 del Codigo Penal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="28" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>3. Conteo de dias</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   El periodo se parte en tramos que no cruzan fin de mes, para que a cada dia se le</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   aplique la tasa vigente en su propio mes. Cada tramo se cuenta como diferencia de</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   fechas (fecha final menos fecha inicial): el dia inicial se cuenta y el dia final</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   no, de modo que ningun dia queda contado dos veces en el paso de un mes al otro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>4. Formula</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Intereses del tramo = Capital x [ (1 + tasa mora E.A.) ^ (dias / 365) - 1 ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Es la conversion de la tasa efectiva anual a su equivalente por el numero exacto de</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   dias del tramo. Los intereses se calculan siempre sobre el capital insoluto: no se</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   capitalizan intereses (prohibicion de anatocismo, art. 2235 C.C. y art. 886 C.Co.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="28" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>5. Codigo de colores</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Azul: dato tomado de fuente externa o suministrado por el usuario (editable).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Amarillo: celda de entrada que el usuario puede modificar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Negro: resultado calculado por formula. Verde: enlace a otra hoja del mismo libro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>6. Advertencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Esta liquidacion es un calculo aritmetico. La tasa efectivamente aplicable depende</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   del titulo, del pacto de las partes y de lo ordenado en el mandamiento de pago; si el</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   titulo pacto una tasa inferior, debe reemplazarse en la hoja Tasas.</t>
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>- Celdas amarillas: unicas editables (capital, fechas y tasa de cada mes). El resto son formulas.</t>
         </is>
       </c>
     </row>

</xml_diff>